<commit_message>
fix gpt-4 vision errors
</commit_message>
<xml_diff>
--- a/sample_statements/sample_jon_doe.xlsx
+++ b/sample_statements/sample_jon_doe.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\Personal_projects\Financial_Analyst_RAG\cursor3\sample_statements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A52C8C9-3E01-48A6-AC5A-46CF586C03FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7CF69E6-00B9-474B-B334-D0F6C402AD29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -227,29 +227,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Closing Balance:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> 2,793.78</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
       <t>Total Credit</t>
     </r>
     <r>
@@ -309,6 +286,29 @@
       <t xml:space="preserve"> 1,000.00</t>
     </r>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Closing Balance:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 1,793.78</t>
+    </r>
+  </si>
 </sst>
 </file>
 
@@ -316,7 +316,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="[$€-2]\ #,##0.00;[Red]\-[$€-2]\ #,##0.00"/>
-    <numFmt numFmtId="170" formatCode="[$€-2]\ #,##0.00"/>
+    <numFmt numFmtId="165" formatCode="[$€-2]\ #,##0.00"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -391,7 +391,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -411,13 +411,10 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="170" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -777,7 +774,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="11" t="s">
         <v>56</v>
       </c>
       <c r="E5" t="s">
@@ -789,8 +786,8 @@
         <v>55</v>
       </c>
       <c r="B6" s="3"/>
-      <c r="C6" s="12" t="s">
-        <v>60</v>
+      <c r="C6" s="11" t="s">
+        <v>59</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" t="s">
@@ -798,22 +795,19 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="11" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="C8" s="11" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="C8" s="12" t="s">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="C9" s="11" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="C9" s="12" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="C10" s="12"/>
     </row>
     <row r="12" spans="1:5" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A12" s="7" t="s">
@@ -822,7 +816,7 @@
       <c r="B12" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="C12" s="12" t="s">
         <v>3</v>
       </c>
       <c r="D12" s="7" t="s">

</xml_diff>